<commit_message>
Daily EOD data and reports for 2026-09-17
</commit_message>
<xml_diff>
--- a/asx_eod_output/Report_XLSX/Report_20260901.xlsx
+++ b/asx_eod_output/Report_XLSX/Report_20260901.xlsx
@@ -538,79 +538,79 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ASM</t>
+          <t>BHP</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>0</v>
+        <v>66.84</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>-1.17</v>
+        <v>0.61</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>-100.00%</t>
+          <t>0.92%</t>
         </is>
       </c>
       <c r="E6" s="3" t="n">
-        <v>57458</v>
+        <v>9000</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>0</v>
+        <v>601560</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>-67225.86</v>
+        <v>5490</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>BHP</t>
+          <t>CAN</t>
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>66.84</v>
+        <v>0.004</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>0.61</v>
+        <v>0</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>0.92%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="E7" s="3" t="n">
-        <v>9000</v>
+        <v>44090</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>601560</v>
+        <v>176.36</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>5490</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CAN</t>
+          <t>CBA</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>0.004</v>
+        <v>159.15</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>0</v>
+        <v>-0.75</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>-0.47%</t>
         </is>
       </c>
       <c r="E8" s="3" t="n">
-        <v>44090</v>
+        <v>0</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>176.36</v>
+        <v>0</v>
       </c>
       <c r="G8" s="4" t="n">
         <v>0</v>
@@ -619,109 +619,109 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CBA</t>
+          <t>CNB</t>
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>159.15</v>
+        <v>0.98</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>-0.75</v>
+        <v>0.015</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>-0.47%</t>
+          <t>1.55%</t>
         </is>
       </c>
       <c r="E9" s="3" t="n">
-        <v>0</v>
+        <v>10000</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>0</v>
+        <v>9800</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>0</v>
+        <v>150</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CNB</t>
+          <t>CSL</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>0.98</v>
+        <v>172.31</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>0.015</v>
+        <v>0.74</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>1.55%</t>
+          <t>0.43%</t>
         </is>
       </c>
       <c r="E10" s="3" t="n">
-        <v>10000</v>
+        <v>4000</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>9800</v>
+        <v>689240</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>150</v>
+        <v>2960</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CSL</t>
+          <t>E25</t>
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>172.31</v>
+        <v>0.27</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>0.74</v>
+        <v>0</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0.43%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="E11" s="3" t="n">
-        <v>4000</v>
+        <v>20000</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>689240</v>
+        <v>5400</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>2960</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>E25</t>
+          <t>EF2</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>0.27</v>
+        <v>19.8</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>0</v>
+        <v>-0.5</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>-2.46%</t>
         </is>
       </c>
       <c r="E12" s="3" t="n">
-        <v>20000</v>
+        <v>3045</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>5400</v>
+        <v>60291</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>0</v>
+        <v>-1522.5</v>
       </c>
     </row>
     <row r="13">
@@ -731,24 +731,24 @@
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>0</v>
+        <v>0.002</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>-0.002</v>
+        <v>0</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>-100.00%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="E13" s="3" t="n">
         <v>700000</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>0</v>
+        <v>1400</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>-1400</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -870,10 +870,10 @@
       <c r="D18" s="5" t="inlineStr"/>
       <c r="E18" s="7" t="inlineStr"/>
       <c r="F18" s="8" t="n">
-        <v>1819347.48</v>
+        <v>1881038.48</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>-47890.92</v>
+        <v>19212.44</v>
       </c>
     </row>
   </sheetData>

</xml_diff>